<commit_message>
feat(F-NAR-019): ATOM-EMO.GES.001-03 Nina dit stop au parc
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-EMO.GES.001-03.xlsx
+++ b/stories/arbres/ATOM-EMO.GES.001-03.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Le câlin du parc</t>
+          <t>Nina dit stop au parc</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>parc</t>
+          <t>parc, toboggan, herbe, soleil, sac, jaune, vent, poussière, marches</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Chouchou, Victorina, maman</t>
+          <t>Nina, Raphaël, papa, maman</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Chouchou joue au parc. Victorina le serre trop fort. Il dit stop, s'éloigne vers maman. Plus tard il reprend un seau de sable tiède.</t>
+          <t>Le soleil tient le jaune. Près du sac, un éclat de toboggan brille. Nina veut glisser, maintenant. Raphaël ouvre les bras, serre trop. Sourire parti, poitrine, maman accroupie. Stop, recule. Merci vécu. Deuxième ruse : un câlin au pied. Un éclat de toboggan tient sur le jaune.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Le portail du parc grince. Le trèfle sent le miel. Le toboggan jaune est chaud au soleil. Un moineau saute sur la clôture. Le banc vert attend à l'ombre. Le sac de maman est dessus. Tu as vu le moineau, Chouchou ? Oui, maman. Il saute. Il a des plumes grises. L'herbe est sèche et douce. En ce moment, Chouchou joue avec Victorina. Ils sont près du banc. Victorina ouvre les bras. Elle fait un gros câlin. Le câlin est trop fort. Chouchou est inquiet. Victorina le serre trop près. Sa poitrine est coincée. Ses épaules montent. Je n'aime pas. C'est trop. Stop. Chouchou recule d'un pas. Il peut s'éloigner. Il s'éloigne vers le banc. Maman est l'adulte sur le banc. Maman, c'était trop. Tu as dit stop. Bravo, Chouchou. Tu t'es éloigné. Tu es venu vers moi. Tu veux ta main dans ma main ? Oui, maman. Chouchou pose sa main dans la main de maman. Il souffle. Ses épaules descendent. Dire stop, c'est permis. On s'éloigne. On va vers un adulte. Plus tard, Victorina joue au bac à sable. Le sable est tiède. Chouchou reste près de maman. Tu veux un seau, maintenant ? Oui. Un seau. Chouchou reprend un seau bleu. Le sable coule entre ses doigts. Il est chaud et un peu mouillé. Chouchou fait une petite colline. Elle est ronde, ta colline. Tu as bien travaillé. Elle est ronde, maman. Un papillon passe près du trèfle. Ses ailes sont jaunes.</t>
+          <t>Le soleil pose une bande chaude sur le jaune. L'herbe sent l'été, au parc. Ça sent bon, papa. Tu le sens, l'herbe, Nina ? Oui, papa. Le toboggan jaune tient le soleil. Une poussière d'été danse au bord. Il est jaune, maman. Tu le vois, le toboggan ? Oui, maman. Près du sac, un éclat de toboggan brille. Il brille, papa. Tu le vois, le petit point ? Oui, un petit point. Maman pose le sac dans l'herbe. Le tissu est chaud, un peu rêche. Il est chaud. Tu veux un coin d'ombre ? Oui. Nina touche le jaune du toboggan. Le plastique est tiède, lisse. Le jaune tient chaud, Nina ? Oui, papa. En ce moment, Nina tient le bord. Ses pieds veulent les marches. Je veux glisser, maintenant ! Sur le toboggan, tout de suite. Le toboggan, là ? Oui, le toboggan. Tes mains tiennent le bord, Nina ? Oui, maman. Raphaël arrive dans l'herbe. Il ouvre les bras tout grand. Nina ! Un câlin ! Je glisse, maintenant ! Nina avance trop vite vers lui. Raphaël la serre contre sa poitrine. Le câlin est trop fort. Oh. Nina connaît le toboggan. Elle veut les marches. Les bras serrent trop près. Viens ! Raphaël serre plus fort, content. Nina ne peut plus bouger. Le sourire de Nina disparaît. Dans sa poitrine, l'air se coince. Ses épaules montent un peu. Maman s'accroupit à la même hauteur. Tu vois Raphaël, Nina ? Oui, maman. Les bras sont trop près, Nina ? Un peu, papa. L'éclat de toboggan tremble, puis tient. Raphaël baisse les yeux. Je ne peux plus, maman. Nina regarde maman.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Le portail du parc grince. Le trèfle sent le miel. Le toboggan jaune est chaud au soleil. Un moineau saute sur la clôture. Le banc vert attend à l'ombre. Le sac de maman est dessus. Tu as vu le moineau, Chouchou ? Oui, maman. Il saute. Il a des plumes grises. L'herbe est sèche et douce. En ce moment, Chouchou joue avec Victorina. Ils sont près du banc. Victorina ouvre les bras. Elle fait un gros câlin. Le câlin est trop fort. Chouchou est inquiet. Victorina le serre trop près. Sa poitrine est coincée. Ses épaules montent. Je n'aime pas. C'est trop. Stop. Chouchou recule d'un pas. Il peut s'éloigner. Il s'éloigne vers le banc. Maman est l'adulte sur le banc. Maman, c'était trop. Tu as dit stop. Bravo, Chouchou. Tu t'es éloigné. Tu es venu vers moi. Tu veux ta main dans ma main ? Oui, maman. Chouchou pose sa main dans la main de maman. Il souffle. Ses épaules descendent. Dire stop, c'est permis. On s'éloigne. On va vers un adulte. Plus tard, Victorina joue au bac à sable. Le sable est tiède. Chouchou reste près de maman. Tu veux un seau, maintenant ? Oui. Un seau. Chouchou reprend un seau bleu. Le sable coule entre ses doigts. Il est chaud et un peu mouillé. Chouchou fait une petite colline. Elle est ronde, ta colline. Tu as bien travaillé. Elle est ronde, maman. Un papillon passe près du trèfle. Ses ailes sont jaunes.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le soleil pose une bande chaude sur le jaune. L'herbe sent l'été, au parc. Ça sent bon, papa. Tu le sens, l'herbe, Nina ? Oui, papa. Le toboggan jaune tient le soleil. Une poussière d'été danse au bord. Il est jaune, maman. Tu le vois, le toboggan ? Oui, maman. Près du sac, un &lt;emphasis level="moderate"&gt;éclat de toboggan&lt;/emphasis&gt; brille. Il brille, papa. Tu le vois, le petit point ? Oui, un petit point. Maman pose le sac dans l'herbe. Le tissu est chaud, un peu rêche. Il est chaud. Tu veux un coin d'ombre ? Oui. Nina touche le jaune du toboggan. Le plastique est tiède, lisse. Le jaune tient chaud, Nina ? Oui, papa. En ce moment, Nina tient le bord. Ses pieds veulent les marches. Je veux glisser, maintenant ! Sur le toboggan, tout de suite. Le toboggan, là ? Oui, le toboggan. Tes mains tiennent le bord, Nina ? Oui, maman. Raphaël arrive dans l'herbe. Il ouvre les bras tout grand. Nina ! Un câlin ! Je glisse, maintenant ! Nina avance trop vite vers lui. Raphaël la serre contre sa poitrine. Le câlin est trop fort. Oh. Nina connaît le toboggan. Elle veut les marches. Les bras serrent trop près. Viens ! Raphaël serre plus fort, content. Nina ne peut plus bouger. Le sourire de Nina disparaît. Dans sa poitrine, l'air se coince. Ses épaules montent un peu. Maman s'accroupit à la même hauteur. Tu vois Raphaël, Nina ? Oui, maman. Les bras sont trop près, Nina ? Un peu, papa. L'éclat de toboggan tremble, puis tient. Raphaël baisse les yeux. Je ne peux plus, maman. Nina regarde maman.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Fatou joue au parc. L'herbe sent l'été. Côme la serre trop fort dans un câlin. Fatou sent sa poitrine coincée. Ses épaules montent. Elle dit : je n'aime pas. C'est trop. Fatou dit : &lt;emphasis&gt;stop&lt;/emphasis&gt;. Elle recule d'un pas. Elle peut s'éloigner. Elle s'éloigne vers le banc. Maman est l'adulte sur le banc. Fatou va vers maman. Elle dit : c'était trop. Maman l'écoute. Fatou pose sa main dans la main de maman. Elle souffle. Ses épaules descendent. Dire stop, c'est permis. On s'éloigne. On va vers un adulte. Plus tard, Côme joue au bac à sable. Fatou reste près de maman. Puis elle reprend un seau. Le sable est tiède. [pause]</t>
+          <t>Le soleil pose une bande chaude sur le jaune. L'herbe sent l'été, au parc. Ça sent bon, papa. Tu le sens, l'herbe, Nina ? Oui, papa. Le toboggan jaune tient le soleil. Une poussière d'été danse au bord. Il est jaune, maman. Tu le vois, le toboggan ? Oui, maman. Près du sac, un &lt;emphasis&gt;éclat de toboggan&lt;/emphasis&gt; brille. Il brille, papa. Tu le vois, le petit point ? Oui, un petit point. Maman pose le sac dans l'herbe. Le tissu est chaud, un peu rêche. Il est chaud. Tu veux un coin d'ombre ? Oui. Nina touche le jaune du toboggan. Le plastique est tiède, lisse. Le jaune tient chaud, Nina ? Oui, papa. En ce moment, Nina tient le bord. Ses pieds veulent les marches. Je veux glisser, maintenant ! Sur le toboggan, tout de suite. Le toboggan, là ? Oui, le toboggan. Tes mains tiennent le bord, Nina ? Oui, maman. Raphaël arrive dans l'herbe. Il ouvre les bras tout grand. Nina ! Un câlin ! Je glisse, maintenant ! Nina avance trop vite vers lui. Raphaël la serre contre sa poitrine. Le câlin est trop fort. Oh. Nina connaît le toboggan. Elle veut les marches. Les bras serrent trop près. Viens ! Raphaël serre plus fort, content. Nina ne peut plus bouger. Le sourire de Nina disparaît. Dans sa poitrine, l'air se coince. Ses épaules montent un peu. Maman s'accroupit à la même hauteur. Tu vois Raphaël, Nina ? Oui, maman. Les bras sont trop près, Nina ? Un peu, papa. L'éclat de toboggan tremble, puis tient. Raphaël baisse les yeux. Je ne peux plus, maman. Nina regarde maman. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,7 +1246,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1254,10 +1254,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.18</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1280,30 +1280,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>stop</t>
+          <t>éclat de toboggan</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1326,62 +1326,71 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis serrement; intensite=2; destinataire=enfant; sous_texte=elle_veut_glisser_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Le portail du parc grince.
-narrateur|Le trèfle sent le miel.
-narrateur|Le toboggan jaune est chaud au soleil.
-narrateur|Un moineau saute sur la clôture.
-narrateur|Le banc vert attend à l'ombre.
-narrateur|Le sac de maman est dessus.
-maman|Tu as vu le moineau, Chouchou ?
-enfant-m|Oui, maman. Il saute.
-maman|Il a des plumes grises.
-narrateur|L'herbe est sèche et douce.
-narrateur|En ce moment, Chouchou joue avec Victorina.
-narrateur|Ils sont près du banc.
-narrateur|Victorina ouvre les bras.
-narrateur|Elle fait un gros câlin.
+          <t>narrateur|Le soleil pose une bande chaude sur le jaune.
+narrateur|L'herbe sent l'été, au parc.
+enfant-f|Ça sent bon, papa.
+papa|Tu le sens, l'herbe, Nina ?
+enfant-f|Oui, papa.
+narrateur|Le toboggan jaune tient le soleil.
+narrateur|Une poussière d'été danse au bord.
+enfant-f|Il est jaune, maman.
+maman|Tu le vois, le toboggan ?
+enfant-f|Oui, maman.
+narrateur|Près du sac, un éclat de toboggan brille.
+enfant-f|Il brille, papa.
+papa|Tu le vois, le petit point ?
+enfant-f|Oui, un petit point.
+narrateur|Maman pose le sac dans l'herbe.
+narrateur|Le tissu est chaud, un peu rêche.
+enfant-f|Il est chaud.
+maman|Tu veux un coin d'ombre ?
+enfant-f|Oui.
+narrateur|Nina touche le jaune du toboggan.
+narrateur|Le plastique est tiède, lisse.
+papa|Le jaune tient chaud, Nina ?
+enfant-f|Oui, papa.
+narrateur|En ce moment, Nina tient le bord.
+narrateur|Ses pieds veulent les marches.
+enfant-f|Je veux glisser, maintenant !
+enfant-f|Sur le toboggan, tout de suite.
+papa|Le toboggan, là ?
+enfant-f|Oui, le toboggan.
+maman|Tes mains tiennent le bord, Nina ?
+enfant-f|Oui, maman.
+narrateur|Raphaël arrive dans l'herbe.
+narrateur|Il ouvre les bras tout grand.
+copain|Nina !
+copain|Un câlin !
+enfant-f|Je glisse, maintenant !
+narrateur|Nina avance trop vite vers lui.
+narrateur|Raphaël la serre contre sa poitrine.
 narrateur|Le câlin est trop fort.
-narrateur|Chouchou est inquiet.
-narrateur|Victorina le serre trop près.
-narrateur|Sa poitrine est coincée.
-narrateur|Ses épaules montent.
-enfant-m|Je n'aime pas.
-enfant-m|C'est trop.
-enfant-m|Stop.
-narrateur|Chouchou recule d'un pas.
-narrateur|Il peut s'éloigner.
-narrateur|Il s'éloigne vers le banc.
-narrateur|Maman est l'adulte sur le banc.
-enfant-m|Maman, c'était trop.
-maman|Tu as dit stop.
-maman|Bravo, Chouchou.
-maman|Tu t'es éloigné.
-maman|Tu es venu vers moi.
-maman|Tu veux ta main dans ma main ?
-enfant-m|Oui, maman.
-narrateur|Chouchou pose sa main dans la main de maman.
-narrateur|Il souffle.
-narrateur|Ses épaules descendent.
-maman|Dire stop, c'est permis.
-maman|On s'éloigne.
-maman|On va vers un adulte.
-narrateur|Plus tard, Victorina joue au bac à sable.
-narrateur|Le sable est tiède.
-narrateur|Chouchou reste près de maman.
-maman|Tu veux un seau, maintenant ?
-enfant-m|Oui. Un seau.
-narrateur|Chouchou reprend un seau bleu.
-narrateur|Le sable coule entre ses doigts.
-narrateur|Il est chaud et un peu mouillé.
-narrateur|Chouchou fait une petite colline.
-maman|Elle est ronde, ta colline.
-maman|Tu as bien travaillé.
-enfant-m|Elle est ronde, maman.
-narrateur|Un papillon passe près du trèfle.
-narrateur|Ses ailes sont jaunes.</t>
+enfant-f|Oh.
+narrateur|Nina connaît le toboggan.
+narrateur|Elle veut les marches.
+narrateur|Les bras serrent trop près.
+copain|Viens !
+narrateur|Raphaël serre plus fort, content.
+narrateur|Nina ne peut plus bouger.
+narrateur|Le sourire de Nina disparaît.
+narrateur|Dans sa poitrine, l'air se coince.
+narrateur|Ses épaules montent un peu.
+narrateur|Maman s'accroupit à la même hauteur.
+maman|Tu vois Raphaël, Nina ?
+enfant-f|Oui, maman.
+papa|Les bras sont trop près, Nina ?
+enfant-f|Un peu, papa.
+narrateur|L'éclat de toboggan tremble, puis tient.
+narrateur|Raphaël baisse les yeux.
+enfant-f|Je ne peux plus, maman.
+narrateur|Nina regarde maman.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
@@ -1413,17 +1422,17 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>C'est trop pour Chouchou. Que dit-il ?</t>
+          <t>C'est trop pour Nina. Que dit-elle ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>C'est trop pour Chouchou. Que dit-il ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;C'est trop pour &lt;emphasis level="moderate"&gt;Nina&lt;/emphasis&gt;. Que dit-elle ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;C'est trop pour Fatou. Que dit-elle ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;C'est trop pour &lt;emphasis&gt;Nina&lt;/emphasis&gt;. Que dit-elle ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1486,7 +1495,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1497,7 +1506,7 @@
         <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.3</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1512,34 +1521,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>Nina</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1554,22 +1567,23 @@
         <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=c_est_trop_que_dit_elle; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|C'est trop pour Chouchou. Que dit-il ?</t>
+          <t>narrateur|C'est trop pour Nina.
+narrateur|Que dit-elle ?</t>
         </is>
       </c>
     </row>
@@ -1596,17 +1610,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Chouchou a dit stop. Il a pu s'éloigner. Il a rejoint maman, l'adulte. Tu as dit le bon mot. Stop. Bravo. Tu restes près du banc ? Oui. Le moineau est encore sur la clôture. Le trèfle sent toujours le miel.</t>
+          <t>Nina veut glisser, tout de suite. Je pars, maintenant ! Elle tire vers les marches. Les bras restent collés. Raphaël serre, sans le vouloir. L'air manque dans sa poitrine. Oh. Le sourire ne revient pas. Nina refuse de rester prise. Stop. Elle recule d'un pas. Les bras s'ouvrent. L'air revient, chaud. Tu veux de la place, Nina ? Maman reste à la même hauteur. Maman, on fait quoi ? On reste un peu, puis on glisse. D'accord. Nina reste un moment, les mains ouvertes. Elle garde un pas d'herbe. Pardon. C'est trop. Raphaël hoche la tête. Nina pose une main sur le sac. Merci, Nina. Papa a vu les deux, dans l'herbe. Le jaune est tiède, sous les doigts. Il est chaud. Papa tend le bord du toboggan. Nina touche. C'est lisse et chaud. Raphaël touche aussi. Le toboggan. Il a des marches, là ? Oui, là. Nina glisse la main sur le jaune. Le plastique est lisse, contre la peau. Tes mains sont au chaud, Nina ? Un peu, maman. Raphaël pose un doigt sur le bord. Jaune. On y va, après ? Le sac est près du toboggan. Oui, maman.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Chouchou a dit stop. Il a pu s'éloigner. Il a rejoint maman, l'adulte. Tu as dit le bon mot. Stop. Bravo. Tu restes près du banc ? Oui. Le moineau est encore sur la clôture. Le trèfle sent toujours le miel.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nina veut glisser, tout de suite. Je pars, maintenant ! Elle tire vers les marches. Les bras restent collés. Raphaël serre, sans le vouloir. L'air manque dans sa poitrine. Oh. Le sourire ne revient pas. Nina refuse de rester prise. &lt;emphasis level="moderate"&gt;Stop&lt;/emphasis&gt;. Elle recule d'un pas. Les bras s'ouvrent. L'air revient, chaud. Tu veux de la place, Nina ? Maman reste à la même hauteur. Maman, on fait quoi ? On reste un peu, puis on glisse. D'accord. Nina reste un moment, les mains ouvertes. Elle garde un pas d'herbe. Pardon. C'est trop. Raphaël hoche la tête. Nina pose une main sur le sac. Merci, Nina. Papa a vu les deux, dans l'herbe. Le jaune est tiède, sous les doigts. Il est chaud. Papa tend le bord du toboggan. Nina touche. C'est lisse et chaud. Raphaël touche aussi. Le toboggan. Il a des marches, là ? Oui, là. Nina glisse la main sur le jaune. Le plastique est lisse, contre la peau. Tes mains sont au chaud, Nina ? Un peu, maman. Raphaël pose un doigt sur le bord. Jaune. On y va, après ? Le sac est près du toboggan. Oui, maman.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Fatou a dit &lt;emphasis&gt;stop&lt;/emphasis&gt;. Elle a pu s'éloigner. Elle rejoint maman, l'adulte. [pause]</t>
+          <t>Nina veut glisser, tout de suite. Je pars, maintenant ! Elle tire vers les marches. Les bras restent collés. Raphaël serre, sans le vouloir. L'air manque dans sa poitrine. Oh. Le sourire ne revient pas. Nina refuse de rester prise. &lt;emphasis&gt;Stop&lt;/emphasis&gt;. Elle recule d'un pas. Les bras s'ouvrent. L'air revient, chaud. Tu veux de la place, Nina ? Maman reste à la même hauteur. Maman, on fait quoi ? On reste un peu, puis on glisse. D'accord. Nina reste un moment, les mains ouvertes. Elle garde un pas d'herbe. Pardon. C'est trop. Raphaël hoche la tête. Nina pose une main sur le sac. Merci, Nina. Papa a vu les deux, dans l'herbe. Le jaune est tiède, sous les doigts. Il est chaud. Papa tend le bord du toboggan. Nina touche. C'est lisse et chaud. Raphaël touche aussi. Le toboggan. Il a des marches, là ? Oui, là. Nina glisse la main sur le jaune. Le plastique est lisse, contre la peau. Tes mains sont au chaud, Nina ? Un peu, maman. Raphaël pose un doigt sur le bord. Jaune. On y va, après ? Le sac est près du toboggan. Oui, maman. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1653,7 +1667,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1661,10 +1675,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.18</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1687,30 +1701,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>stop</t>
+          <t>Stop</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1719,10 +1733,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1735,21 +1749,55 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis air_qui_revient; intensite=2; destinataire=enfant; sous_texte=elle_dit_stop_elle_recule; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Chouchou a dit stop.
-narrateur|Il a pu s'éloigner.
-narrateur|Il a rejoint maman, l'adulte.
-maman|Tu as dit le bon mot.
-maman|Stop.
-maman|Bravo.
-maman|Tu restes près du banc ?
-enfant-m|Oui.
-narrateur|Le moineau est encore sur la clôture.
-narrateur|Le trèfle sent toujours le miel.</t>
+          <t>narrateur|Nina veut glisser, tout de suite.
+enfant-f|Je pars, maintenant !
+narrateur|Elle tire vers les marches.
+narrateur|Les bras restent collés.
+narrateur|Raphaël serre, sans le vouloir.
+narrateur|L'air manque dans sa poitrine.
+enfant-f|Oh.
+narrateur|Le sourire ne revient pas.
+narrateur|Nina refuse de rester prise.
+enfant-f|Stop.
+narrateur|Elle recule d'un pas.
+narrateur|Les bras s'ouvrent.
+narrateur|L'air revient, chaud.
+maman|Tu veux de la place, Nina ?
+narrateur|Maman reste à la même hauteur.
+enfant-f|Maman, on fait quoi ?
+maman|On reste un peu, puis on glisse.
+enfant-f|D'accord.
+narrateur|Nina reste un moment, les mains ouvertes.
+narrateur|Elle garde un pas d'herbe.
+copain|Pardon.
+enfant-f|C'est trop.
+narrateur|Raphaël hoche la tête.
+narrateur|Nina pose une main sur le sac.
+papa|Merci, Nina.
+narrateur|Papa a vu les deux, dans l'herbe.
+maman|Le jaune est tiède, sous les doigts.
+enfant-f|Il est chaud.
+narrateur|Papa tend le bord du toboggan.
+narrateur|Nina touche.
+narrateur|C'est lisse et chaud.
+narrateur|Raphaël touche aussi.
+enfant-f|Le toboggan.
+papa|Il a des marches, là ?
+enfant-f|Oui, là.
+narrateur|Nina glisse la main sur le jaune.
+narrateur|Le plastique est lisse, contre la peau.
+maman|Tes mains sont au chaud, Nina ?
+enfant-f|Un peu, maman.
+narrateur|Raphaël pose un doigt sur le bord.
+copain|Jaune.
+enfant-f|On y va, après ?
+maman|Le sac est près du toboggan.
+enfant-f|Oui, maman.</t>
         </is>
       </c>
     </row>
@@ -1776,17 +1824,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Chouchou reste près du banc vert. Maman lui parle tout bas. Ton corps a parlé. Ta poitrine était coincée. Tu as écouté. Tu es plus calme, maintenant ? Oui, maman. Le seau bleu est plein de sable tiède. Chouchou le pose près du banc. Il souffle encore une fois. Le toboggan jaune brille encore. Chouchou reste près de maman. On peut regarder le moineau. Il est encore là.</t>
+          <t>Ils restent près du toboggan. Nina pose un pied sur la marche. On y va ensemble ! Je glisse, maintenant ! Raphaël ouvre les bras trop vite. Il la serre pour monter. Oh. Nina avance les pieds, trop vite. Puis elle s'arrête net. Nina refuse de rester prise, cette fois. Sa poitrine se serre, puis s'ouvre. Stop. Elle recule d'un pas. Personne ne serre plus. Elle observe le jaune, un instant. Elle écoute le vent du parc. Au pied, un éclat de toboggan luit. Là, sur le jaune. Tu montes après, Raphaël ? Raphaël ne serre plus. Il tient le bord, sans coller. Après toi. Nina recule un peu, sans se presser. Raphaël pose les mains, plus lentement. Le plastique est lisse et tiède. Tu la vois, la marche ? Oui, papa. Le sac est près du jaune ? Oui, maman. Le toboggan tient contre le soleil. Nina pose une main sur le bord. Raphaël pose la suivante. Le jaune tient, Nina ? Oui, papa. Le vent passe sur l'herbe. Il chatouille les genoux.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Chouchou reste près du banc vert. Maman lui parle tout bas. Ton corps a parlé. Ta poitrine était coincée. Tu as écouté. Tu es plus calme, maintenant ? Oui, maman. Le seau bleu est plein de sable tiède. Chouchou le pose près du banc. Il souffle encore une fois. Le toboggan jaune brille encore. Chouchou reste près de maman. On peut regarder le moineau. Il est encore là.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Ils restent près du toboggan. Nina pose un pied sur la marche. On y va ensemble ! Je glisse, maintenant ! Raphaël ouvre les bras trop vite. Il la serre pour monter. Oh. Nina avance les pieds, trop vite. Puis elle s'arrête net. Nina refuse de rester prise, cette fois. Sa poitrine se serre, puis s'ouvre. Stop. Elle recule d'un pas. Personne ne serre plus. Elle observe le jaune, un instant. Elle écoute le vent du parc. Au pied, un &lt;emphasis level="moderate"&gt;éclat de toboggan&lt;/emphasis&gt; luit. Là, sur le jaune. Tu montes après, Raphaël ? Raphaël ne serre plus. Il tient le bord, sans coller. Après toi. Nina recule un peu, sans se presser. Raphaël pose les mains, plus lentement. Le plastique est lisse et tiède. Tu la vois, la marche ? Oui, papa. Le sac est près du jaune ? Oui, maman. Le toboggan tient contre le soleil. Nina pose une main sur le bord. Raphaël pose la suivante. Le jaune tient, Nina ? Oui, papa. Le vent passe sur l'herbe. Il chatouille les genoux.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Fatou reste près du banc. Maman lui parle tout bas. [pause]</t>
+          <t>Ils restent près du toboggan. Nina pose un pied sur la marche. On y va ensemble ! Je glisse, maintenant ! Raphaël ouvre les bras trop vite. Il la serre pour monter. Oh. Nina avance les pieds, trop vite. Puis elle s'arrête net. Nina refuse de rester prise, cette fois. Sa poitrine se serre, puis s'ouvre. Stop. Elle recule d'un pas. Personne ne serre plus. Elle observe le jaune, un instant. Elle écoute le vent du parc. Au pied, un &lt;emphasis&gt;éclat de toboggan&lt;/emphasis&gt; luit. Là, sur le jaune. Tu montes après, Raphaël ? Raphaël ne serre plus. Il tient le bord, sans coller. Après toi. Nina recule un peu, sans se presser. Raphaël pose les mains, plus lentement. Le plastique est lisse et tiède. Tu la vois, la marche ? Oui, papa. Le sac est près du jaune ? Oui, maman. Le toboggan tient contre le soleil. Nina pose une main sur le bord. Raphaël pose la suivante. Le jaune tient, Nina ? Oui, papa. Le vent passe sur l'herbe. Il chatouille les genoux. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1833,7 +1881,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1841,10 +1889,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.18</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1865,28 +1913,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>éclat de toboggan</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1895,10 +1947,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1909,23 +1961,49 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=calin_au_pied_elle_recule_encore; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Chouchou reste près du banc vert.
-narrateur|Maman lui parle tout bas.
-maman|Ton corps a parlé.
-maman|Ta poitrine était coincée.
-maman|Tu as écouté.
-maman|Tu es plus calme, maintenant ?
-enfant-m|Oui, maman.
-narrateur|Le seau bleu est plein de sable tiède.
-narrateur|Chouchou le pose près du banc.
-narrateur|Il souffle encore une fois.
-narrateur|Le toboggan jaune brille encore.
-narrateur|Chouchou reste près de maman.
-maman|On peut regarder le moineau.
-enfant-m|Il est encore là.</t>
+          <t>narrateur|Ils restent près du toboggan.
+narrateur|Nina pose un pied sur la marche.
+copain|On y va ensemble !
+enfant-f|Je glisse, maintenant !
+narrateur|Raphaël ouvre les bras trop vite.
+narrateur|Il la serre pour monter.
+enfant-f|Oh.
+narrateur|Nina avance les pieds, trop vite.
+narrateur|Puis elle s'arrête net.
+narrateur|Nina refuse de rester prise, cette fois.
+narrateur|Sa poitrine se serre, puis s'ouvre.
+enfant-f|Stop.
+narrateur|Elle recule d'un pas.
+narrateur|Personne ne serre plus.
+narrateur|Elle observe le jaune, un instant.
+narrateur|Elle écoute le vent du parc.
+narrateur|Au pied, un éclat de toboggan luit.
+enfant-f|Là, sur le jaune.
+enfant-f|Tu montes après, Raphaël ?
+narrateur|Raphaël ne serre plus.
+narrateur|Il tient le bord, sans coller.
+copain|Après toi.
+narrateur|Nina recule un peu, sans se presser.
+narrateur|Raphaël pose les mains, plus lentement.
+narrateur|Le plastique est lisse et tiède.
+papa|Tu la vois, la marche ?
+enfant-f|Oui, papa.
+maman|Le sac est près du jaune ?
+enfant-f|Oui, maman.
+narrateur|Le toboggan tient contre le soleil.
+narrateur|Nina pose une main sur le bord.
+narrateur|Raphaël pose la suivante.
+papa|Le jaune tient, Nina ?
+enfant-f|Oui, papa.
+maman|Le vent passe sur l'herbe.
+enfant-f|Il chatouille les genoux.</t>
         </is>
       </c>
     </row>
@@ -1952,17 +2030,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>J'ai dit stop. Je me suis éloigné. Je suis allé vers maman. Bravo.</t>
+          <t>Ils restent près du jaune. Le toboggan est à toi, Nina ? Oui, maman. Tu souffles un peu ? Oui, papa. Nina souffle, un filet d'air. L'herbe sent bon. Tu le sens, le parc ? Oui, maman. La glisse reste un peu, chaude. Elle a tenu, sous les mains. Toboggan. L'herbe est chaude, sous les mains. Le jaune fait une ombre ronde. On glisse, après. Un éclat de toboggan tient sur le jaune.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>J'ai dit stop. Je me suis éloigné. Je suis allé vers maman. Bravo.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent près du jaune. Le toboggan est à toi, Nina ? Oui, maman. Tu souffles un peu ? Oui, papa. Nina souffle, un filet d'air. L'herbe sent bon. Tu le sens, le parc ? Oui, maman. La glisse reste un peu, chaude. Elle a tenu, sous les mains. Toboggan. L'herbe est chaude, sous les mains. Le jaune fait une ombre ronde. On glisse, après. Un &lt;emphasis level="moderate"&gt;éclat de toboggan&lt;/emphasis&gt; tient sur le jaune.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent près du jaune. Le toboggan est à toi, Nina ? Oui, maman. Tu souffles un peu ? Oui, papa. Nina souffle, un filet d'air. L'herbe sent bon. Tu le sens, le parc ? Oui, maman. La glisse reste un peu, chaude. Elle a tenu, sous les mains. Toboggan. L'herbe est chaude, sous les mains. Le jaune fait une ombre ronde. On glisse, après. Un &lt;emphasis&gt;éclat de toboggan&lt;/emphasis&gt; tient sur le jaune.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2009,7 +2087,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2017,10 +2095,10 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.26</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2029,12 +2107,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2043,17 +2121,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de toboggan</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2062,11 +2144,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2075,27 +2157,43 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_air_libre; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_jaune; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-m|J'ai dit stop.
-enfant-m|Je me suis éloigné.
-enfant-m|Je suis allé vers maman.
-maman|Bravo.</t>
+          <t>narrateur|Ils restent près du jaune.
+maman|Le toboggan est à toi, Nina ?
+enfant-f|Oui, maman.
+papa|Tu souffles un peu ?
+enfant-f|Oui, papa.
+narrateur|Nina souffle, un filet d'air.
+enfant-f|L'herbe sent bon.
+maman|Tu le sens, le parc ?
+enfant-f|Oui, maman.
+papa|La glisse reste un peu, chaude.
+enfant-f|Elle a tenu, sous les mains.
+copain|Toboggan.
+narrateur|L'herbe est chaude, sous les mains.
+narrateur|Le jaune fait une ombre ronde.
+enfant-f|On glisse, après.
+narrateur|Un éclat de toboggan tient sur le jaune.</t>
         </is>
       </c>
     </row>
@@ -2116,7 +2214,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2173,6 +2271,13 @@
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>